<commit_message>
GITBOOK-20: Upload edited excel
</commit_message>
<xml_diff>
--- a/docs/0OMsoqOg9GiJ2xusVHMv/.gitbook/assets/IO - Template servizi - Alloggi sociali.xlsx
+++ b/docs/0OMsoqOg9GiJ2xusVHMv/.gitbook/assets/IO - Template servizi - Alloggi sociali.xlsx
@@ -827,7 +827,7 @@
         <rFont val="Titillium Web"/>
       </rPr>
       <t xml:space="preserve">
-Puoi pagare direttamente in app premendo “Vedi Avviso”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
+Puoi pagare direttamente in app premendo “Paga”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
 Se hai già provveduto a pagare l'avviso, ignora questo messaggio.
 Per maggiori informazioni o per richiedere assistenza, contattaci tramite i canali che trovi nella scheda servizio.
 In fase di pagamento, se previsto dall'ente, l'importo riportato nel messaggio potrebbe subire variazioni.</t>
@@ -1460,8 +1460,8 @@
         <rFont val="Titillium Web"/>
       </rPr>
       <t xml:space="preserve">
-Puoi pagare direttamente in app premendo “Vedi Avviso”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
-Se hai già provveduto a pagare l'avviso ignora questo messaggio.
+Puoi pagare direttamente in app premendo “Vedi Avviso”, oppure tramite tutti i canali di Puoi pagare direttamente in app premendo “Paga”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
+Se hai già provveduto a pagare l'avviso, ignora questo messaggio.
 Per maggiori informazioni o per richiedere assistenza, contattaci tramite i canali che trovi nella scheda servizio.
 In fase di pagamento, se previsto dall'ente, l'importo riportato nel messaggio potrebbe subire variazioni.</t>
     </r>
@@ -1531,7 +1531,7 @@
     <t>Disdici appuntamento</t>
   </si>
   <si>
-    <t>Vedi Avviso</t>
+    <t>Paga (inserito automaticamente dall'app se il messaggio prevede un avviso di pagamento pagoPA)</t>
   </si>
   <si>
     <t>Accedi al portale</t>

</xml_diff>